<commit_message>
reformulation + intent step, updated mongo storage, conversation history upgrades
</commit_message>
<xml_diff>
--- a/querySparql.xlsx
+++ b/querySparql.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzofilitti/Desktop/SparqlAgent/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAE9014E-72B7-1748-8E48-EF1EBE0F2715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09F82F62-29F9-4947-AA89-1F6E931BAF4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16780" xr2:uid="{7EA1D7AC-A08B-ED4C-963B-D0B97934D44B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="231">
   <si>
     <t>question</t>
   </si>
@@ -1627,6 +1627,225 @@
   </si>
   <si>
     <t xml:space="preserve">show me examples of verbs of the fourth conjugation </t>
+  </si>
+  <si>
+    <t>SELECT ?lemma ?label WHERE {
+  ?lemma a lila:Lemma ;
+         lila:hasPOS lila:noun ;
+         lila:hasInflectionType lila:n1 ;
+         lila:hasGender lila:feminine ;
+         rdfs:label ?label .
+} LIMIT 15</t>
+  </si>
+  <si>
+    <t>Can you list 15 first declension feminine nouns?</t>
+  </si>
+  <si>
+    <t>How many verbs are there for each conjugation type?</t>
+  </si>
+  <si>
+    <t>SELECT ?conjugation (COUNT(?verb) AS ?count) WHERE {
+  ?verb a lila:Lemma ;
+        lila:hasPOS lila:verb ;
+        lila:hasInflectionType ?conjugation .
+}
+GROUP BY ?conjugation
+ORDER BY DESC(?count)</t>
+  </si>
+  <si>
+    <t>SELECT ?lemmaWrittenRep ?definition WHERE {
+  &lt;http://lila-erc.eu/data/lexicalResources/LatinPortuguese/Velez/Lexicon&gt; lime:entry ?lexentry .
+  ?lexentry ontolex:canonicalForm ?lemma ;
+            ontolex:sense ?sense .
+  ?sense &lt;http://www.w3.org/2004/02/skos#definition&gt; ?definition .
+  ?lemma ontolex:writtenRep ?lemmaWrittenRep .
+  FILTER(regex(?definition, "amor", "i"))
+}
+ORDER BY ?lemmaWrittenRep</t>
+  </si>
+  <si>
+    <t>Find lemmas in the Velez dictionary whose definition contains the word "amor".</t>
+  </si>
+  <si>
+    <t>Show me lemmas that are present in the Lewis &amp; Short dictionary but not in the Velez dictionary.</t>
+  </si>
+  <si>
+    <t>SELECT DISTINCT ?lemma ?lemmaLabel WHERE {
+  ?le_ls ontolex:canonicalForm ?lemma .
+  &lt;http://lila-erc.eu/data/lexicalResources/LewisShort/Lexicon&gt; lime:entry ?le_ls .
+  ?lemma rdfs:label ?lemmaLabel .
+  MINUS {
+    ?le_velez ontolex:canonicalForm ?lemma .
+    &lt;http://lila-erc.eu/data/lexicalResources/LatinPortuguese/Velez/Lexicon&gt; lime:entry ?le_velez .
+  }
+}
+ORDER BY ?lemmaLabel
+LIMIT 100</t>
+  </si>
+  <si>
+    <t>What are the comparative and superlative forms of adjectives? Show me 10 examples.</t>
+  </si>
+  <si>
+    <t>SELECT ?adj ?label ?degreeLabel WHERE {
+  VALUES ?degree { lila:comparative lila:superlative }
+  ?adj a lila:Lemma ;
+       lila:hasPOS lila:adjective ;
+       lila:hasDegree ?degree ;
+       rdfs:label ?label .
+  ?degree rdfs:label ?degreeLabel .
+}
+LIMIT 10</t>
+  </si>
+  <si>
+    <t>SELECT ?authorName (COUNT(?doc) as ?documentCount)
+WHERE {
+  ?doc a powla:Document ;
+       dcterms:creator ?author .
+  ?author rdfs:label ?authorName .
+}
+GROUP BY ?authorName
+ORDER BY DESC(?documentCount)</t>
+  </si>
+  <si>
+    <t>Count the number of documents for each author in the knowledge base.</t>
+  </si>
+  <si>
+    <t>Find all verbs that have a reconstructed Proto-Indo-European etymology.</t>
+  </si>
+  <si>
+    <t>SELECT DISTINCT ?lemma ?lemmaLabel ?pieForm WHERE {
+  ?lemma lila:hasPOS lila:verb ;
+         rdfs:label ?lemmaLabel .
+  ?le a ontolex:LexicalEntry ;
+      ontolex:canonicalForm ?lemma ;
+      lemonEty:etymology ?ety .
+  ?ety lemonEty:etymon ?etymon .
+  ?etymon lime:language "PIE" ;
+          rdfs:label ?pieForm .
+}
+ORDER BY ?lemmaLabel
+LIMIT 20</t>
+  </si>
+  <si>
+    <t>SELECT ?lemma ?label WHERE {
+  ?lemma lila:hasPrefix &lt;http://lila-erc.eu/data/id/prefix/12&gt; ; # Corresponds to "con-"
+         rdfs:label ?label .
+}
+LIMIT 20</t>
+  </si>
+  <si>
+    <t>Show me 20 lemmas that are formed with the prefix "con-".</t>
+  </si>
+  <si>
+    <t>SELECT ?prefixLabel (COUNT(DISTINCT ?lemma) AS ?lemmaCount)
+WHERE {
+  ?lemma lila:hasPrefix ?prefix .
+  ?prefix rdfs:label ?prefixLabel .
+}
+GROUP BY ?prefixLabel
+ORDER BY DESC(?lemmaCount)</t>
+  </si>
+  <si>
+    <t>Count how many lemmas are associated with each prefix, showing the most common ones first.</t>
+  </si>
+  <si>
+    <t>SELECT ?tokenLabel ?lemmaLabel WHERE {
+  &lt;http://lila-erc.eu/data/lexicalResources/LatinAffectus/Lexicon&gt; lime:entry ?lexentry .
+  ?lexentry ontolex:canonicalForm ?lemma ;
+            ontolex:sense [ marl:hasPolarity marl:Positive ] .
+  ?lemma rdfs:label ?lemmaLabel .
+  ?token lila:hasLemma ?lemma ;
+         rdfs:label ?tokenLabel .
+  ?token powla:hasLayer/powla:hasDocument/^powla:hasSubDocument &lt;http://lila-erc.eu/data/corpora/UDante/id/corpus&gt; .
+}
+LIMIT 50</t>
+  </si>
+  <si>
+    <t>Find tokens in Dante's works that correspond to lemmas with a positive emotional polarity.</t>
+  </si>
+  <si>
+    <t>SELECT ?lemmaLabel ?suffixLabel WHERE {
+  ?lemma a lila:Lemma ;
+         lila:hasInflectionType lila:n3 ;
+         rdfs:label ?lemmaLabel .
+  OPTIONAL {
+    ?lemma lila:hasSuffix ?suffix .
+    ?suffix rdfs:label ?suffixLabel .
+  }
+}
+LIMIT 100</t>
+  </si>
+  <si>
+    <t>Show me all third declension nouns and, if they have one, list their associated suffix.</t>
+  </si>
+  <si>
+    <t>SELECT DISTINCT ?lemma ?lemmaLabel WHERE {
+  ?token lila:hasLemma ?lemma .
+  ?token powla:hasLayer/powla:hasDocument/^powla:hasSubDocument &lt;http://lila-erc.eu/data/corpora/Lasla/id/corpus&gt; .
+  ?lemma rdfs:label ?lemmaLabel .
+  MINUS {
+    { ?ls_le ontolex:canonicalForm ?lemma . &lt;http://lila-erc.eu/data/lexicalResources/LewisShort/Lexicon&gt; lime:entry ?ls_le . }
+    UNION
+    { ?velez_le ontolex:canonicalForm ?lemma . &lt;http://lila-erc.eu/data/lexicalResources/LatinPortuguese/Velez/Lexicon&gt; lime:entry ?velez_le . }
+  }
+}
+LIMIT 100</t>
+  </si>
+  <si>
+    <t>List lemmas from the LASLA corpus that have no entry in either the Lewis &amp; Short or Velez dictionaries.</t>
+  </si>
+  <si>
+    <t>SELECT ?degreeLabel (COUNT(?adj) AS ?count) WHERE {
+  ?adj a lila:Lemma ;
+       lila:hasPOS lila:adjective ;
+       lila:hasDegree ?degree .
+  ?degree rdfs:label ?degreeLabel .
+}
+GROUP BY ?degreeLabel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Count the number of adjectives for each degree (positive, comparative, superlative).
+</t>
+  </si>
+  <si>
+    <t>SELECT ?lemma ?label WHERE {
+  ?lemma lila:hasPOS lila:proper_noun ;
+         lila:hasGender lila:masculine ;
+         rdfs:label ?label .
+}
+LIMIT 20</t>
+  </si>
+  <si>
+    <t>Find 20 proper nouns that are masculine.</t>
+  </si>
+  <si>
+    <t>SELECT ?lemmaLabel (COUNT(?sense) AS ?senseCount) WHERE {
+  &lt;http://lila-erc.eu/data/lexicalResources/LewisShort/Lexicon&gt; lime:entry ?le .
+  ?le ontolex:canonicalForm ?lemma ;
+      ontolex:sense ?sense .
+  ?lemma rdfs:label ?lemmaLabel .
+}
+GROUP BY ?lemma ?lemmaLabel
+HAVING (COUNT(?sense) &gt; 5)
+ORDER BY DESC(?senseCount)</t>
+  </si>
+  <si>
+    <t>Which lemmas in the Lewis &amp; Short dictionary have more than 5 distinct senses?</t>
+  </si>
+  <si>
+    <t>SELECT ?tokenLabel ?lemmaLabel WHERE {
+  ?le a ontolex:LexicalEntry ;
+      ontolex:canonicalForm ?lemma .
+  &lt;http://lila-erc.eu/data/lexicalResources/IGVLL/Lexicon&gt; lime:entry ?le .
+  ?lemma rdfs:label ?lemmaLabel .
+  ?token lila:hasLemma ?lemma ;
+         rdfs:label ?tokenLabel .
+  ?token powla:hasLayer/powla:hasDocument/^powla:hasSubDocument &lt;http://lila-erc.eu/data/corpora/CLaSSES/id/corpus&gt; .
+}
+LIMIT 50</t>
+  </si>
+  <si>
+    <t>Find occurrences in the CLaSSES corpus of lemmas that have a known Greek etymology</t>
   </si>
 </sst>
 </file>
@@ -2013,7 +2232,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1300A24D-80E3-9B4F-82C4-C9F4C7D1290C}">
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36.6640625" style="4" customWidth="1"/>
@@ -2263,7 +2482,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>187</v>
       </c>
@@ -2274,7 +2493,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="238" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" ht="272" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>186</v>
       </c>
@@ -2307,7 +2526,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>186</v>
       </c>
@@ -2406,7 +2625,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
         <v>186</v>
       </c>
@@ -2417,7 +2636,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>186</v>
       </c>
@@ -2494,7 +2713,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>186</v>
       </c>
@@ -2538,7 +2757,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
         <v>186</v>
       </c>
@@ -2560,7 +2779,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>191</v>
       </c>
@@ -2681,7 +2900,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
         <v>186</v>
       </c>
@@ -2692,7 +2911,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
         <v>186</v>
       </c>
@@ -3053,6 +3272,182 @@
       </c>
       <c r="C94" s="3" t="s">
         <v>197</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" ht="119" x14ac:dyDescent="0.2">
+      <c r="A95" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C95" s="3" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" ht="119" x14ac:dyDescent="0.2">
+      <c r="A96" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C96" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" ht="170" x14ac:dyDescent="0.2">
+      <c r="A97" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" ht="238" x14ac:dyDescent="0.2">
+      <c r="A98" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="C98" s="3" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" ht="153" x14ac:dyDescent="0.2">
+      <c r="A99" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="C99" s="3" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" ht="136" x14ac:dyDescent="0.2">
+      <c r="A100" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="C100" s="3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" ht="204" x14ac:dyDescent="0.2">
+      <c r="A101" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B101" t="s">
+        <v>211</v>
+      </c>
+      <c r="C101" s="3" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" ht="102" x14ac:dyDescent="0.2">
+      <c r="A102" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="C102" s="3" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" ht="119" x14ac:dyDescent="0.2">
+      <c r="A103" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C103" s="3" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" ht="204" x14ac:dyDescent="0.2">
+      <c r="A104" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" ht="170" x14ac:dyDescent="0.2">
+      <c r="A105" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" ht="255" x14ac:dyDescent="0.2">
+      <c r="A106" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" ht="119" x14ac:dyDescent="0.2">
+      <c r="A107" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B107" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" ht="102" x14ac:dyDescent="0.2">
+      <c r="A108" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" ht="170" x14ac:dyDescent="0.2">
+      <c r="A109" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" ht="204" x14ac:dyDescent="0.2">
+      <c r="A110" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: evaluator tool, new prompts, simplified parser
</commit_message>
<xml_diff>
--- a/querySparql.xlsx
+++ b/querySparql.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzofilitti/Desktop/SparqlAgent/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09F82F62-29F9-4947-AA89-1F6E931BAF4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D04E2B2C-988B-074F-B465-6692ECB79DF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16780" xr2:uid="{7EA1D7AC-A08B-ED4C-963B-D0B97934D44B}"/>
+    <workbookView xWindow="20" yWindow="760" windowWidth="29400" windowHeight="16780" xr2:uid="{7EA1D7AC-A08B-ED4C-963B-D0B97934D44B}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="263">
   <si>
     <t>question</t>
   </si>
@@ -1727,13 +1727,6 @@
 LIMIT 20</t>
   </si>
   <si>
-    <t>SELECT ?lemma ?label WHERE {
-  ?lemma lila:hasPrefix &lt;http://lila-erc.eu/data/id/prefix/12&gt; ; # Corresponds to "con-"
-         rdfs:label ?label .
-}
-LIMIT 20</t>
-  </si>
-  <si>
     <t>Show me 20 lemmas that are formed with the prefix "con-".</t>
   </si>
   <si>
@@ -1846,6 +1839,117 @@
   </si>
   <si>
     <t>Find occurrences in the CLaSSES corpus of lemmas that have a known Greek etymology</t>
+  </si>
+  <si>
+    <t>SELECT ?suffixLabel ?type WHERE { ?lemma lila:hasPOS lila:verb ; lila:hasSuffix ?suffix . ?suffix rdfs:label ?suffixLabel ; a ?type . } LIMIT 5</t>
+  </si>
+  <si>
+    <t>List 5 suffixes that attach to verbs and their type.</t>
+  </si>
+  <si>
+    <t>SELECT (COUNT(?lexResource) AS ?count) WHERE { ?lexResource a lime:Lexicon ; dcterms:title ?title . FILTER (CONTAINS(?title, "Dictionary")) }</t>
+  </si>
+  <si>
+    <t>How many lexical resources contain the word "Dictionary" in the title?</t>
+  </si>
+  <si>
+    <t>SELECT ?label WHERE { ?adjective a lila:Lemma ; lila:hasPOS lila:adjective ; lila:hasDegree lila:positive ; rdfs:label ?label . } LIMIT 10</t>
+  </si>
+  <si>
+    <t>Find 10 adjectives in the positive degree.</t>
+  </si>
+  <si>
+    <t>SELECT ?degreeLabel WHERE { ?adjective rdfs:label "magnus" ; lila:hasPOS lila:adjective ; lila:hasDegree ?degree . ?degree rdfs:label ?degreeLabel . }</t>
+  </si>
+  <si>
+    <t>What is the degree of the adjectives with the label "magnus"?</t>
+  </si>
+  <si>
+    <t>SELECT (COUNT(DISTINCT ?lemma) AS ?count) WHERE { &lt;http://lila-erc.eu/data/lexicalResources/LewisShort/Lexicon&gt; lime:entry ?entry . ?entry ontolex:canonicalForm ?lemma . }</t>
+  </si>
+  <si>
+    <t>Count the lemmas associated with the lexical resource "Lewis &amp; Short Dictionary".</t>
+  </si>
+  <si>
+    <t>SELECT ?label WHERE { ?lemma a lila:Lemma ; lila:hasGender lila:feminine ; rdfs:label ?label . } LIMIT 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">List 10 lemmas that have feminine gender </t>
+  </si>
+  <si>
+    <t>SELECT ?prefixLabel (COUNT(?prefix) AS ?count) WHERE { ?lemma lila:hasPrefix ?prefix . ?prefix rdfs:label ?prefixLabel . } GROUP BY ?prefixLabel ORDER BY DESC(?count) LIMIT 5</t>
+  </si>
+  <si>
+    <t>What are the 5 most frequently used prefixes?</t>
+  </si>
+  <si>
+    <t>SELECT (COUNT(DISTINCT ?suffix) AS ?count) WHERE { ?lemma lila:hasPrefix ?suffix}</t>
+  </si>
+  <si>
+    <t>Count the total number of distinct suffixes recorded.</t>
+  </si>
+  <si>
+    <t>SELECT (COUNT(?entry) AS ?count) WHERE { &lt;http://lila-erc.eu/data/lexicalResources/LewisShort/Lexicon&gt; lime:entry ?entry . }</t>
+  </si>
+  <si>
+    <t>How many lexical entries are in the "Lewis &amp; Short Dictionary"?</t>
+  </si>
+  <si>
+    <t>SELECT ?label WHERE { ?adjective a lila:Lemma ; lila:hasPOS lila:adjective ; lila:hasDegree lila:comparative ; rdfs:label ?label . } LIMIT 5</t>
+  </si>
+  <si>
+    <t>Find 5 adjectives that have a comparative degree.</t>
+  </si>
+  <si>
+    <t>SELECT (COUNT(?properNoun) AS ?count) WHERE { ?properNoun a lila:Lemma ; lila:hasPOS lila:proper_noun ; lila:hasGender lila:feminine . }</t>
+  </si>
+  <si>
+    <t>Count the number of proper nouns that are feminine.</t>
+  </si>
+  <si>
+    <t>SELECT ?label WHERE { ?lemma a lila:Lemma ; rdfs:label ?label . FILTER (STRSTARTS(?label, "p")) } limit 20</t>
+  </si>
+  <si>
+    <t>Find 20 lemmas whose label starts with the letter 'P'.</t>
+  </si>
+  <si>
+    <t>SELECT (COUNT(DISTINCT ?degree) AS ?count) WHERE { ?adjective a lila:Lemma ; lila:hasPOS lila:adjective ; lila:hasDegree ?degree . }</t>
+  </si>
+  <si>
+    <t>Count the total number of unique degrees (positive, comparative, superlative) in the KB.</t>
+  </si>
+  <si>
+    <t>SELECT ?posLabel (COUNT(?lemma) AS ?count) WHERE { ?lemma a lila:Lemma ; lila:hasPOS ?pos . ?pos rdfs:label ?posLabel . } GROUP BY ?posLabel ORDER BY DESC(?count)</t>
+  </si>
+  <si>
+    <t>Group lemmas by Part-of-Speech and count how many exist for each POS.</t>
+  </si>
+  <si>
+    <t>SELECT ?label ?definition WHERE { ?entry ontolex:canonicalForm ?noun . ?noun a lila:Lemma ; lila:hasPOS lila:noun ; rdfs:label ?label . ?entry ontolex:sense ?sense . ?sense skos:definition ?definition . FILTER (CONTAINS(?definition, "animal")) } LIMIT 5</t>
+  </si>
+  <si>
+    <t>List 5 nouns with an associated definition that includes the word "animal".</t>
+  </si>
+  <si>
+    <t>SELECT ?lemma ?label WHERE {
+  ?lemma lila:hasPrefix &lt;http://lila-erc.eu/data/id/prefix/12&gt; ; 
+         rdfs:label ?label .
+}
+LIMIT 20</t>
+  </si>
+  <si>
+    <t>What are the documents in the Lasla Corpus that contain the highest number of tokens?</t>
+  </si>
+  <si>
+    <t>SELECT distinct ?corpus ?layer ?document (count(?token) as ?tokenCount) WHERE {
+  ?corpus a powla:Corpus;
+          dc:title "Lasla Corpus";
+          powla:hasSubDocument ?document.
+  ?layer a powla:DocumentLayer;
+          powla:hasDocument ?document.
+  ?token powla:hasLayer ?layer;
+		a powla:Terminal
+} order by desc(?tokenCount) limit 10</t>
   </si>
 </sst>
 </file>
@@ -1881,23 +1985,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -2232,1225 +2328,1402 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1300A24D-80E3-9B4F-82C4-C9F4C7D1290C}">
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C126"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="36.6640625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="27.1640625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="36.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="27.1640625" style="2" customWidth="1"/>
     <col min="3" max="3" width="64.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="51" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="68" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="1" t="s">
         <v>173</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="85" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="1" t="s">
         <v>175</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="68" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="1" t="s">
         <v>177</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="85" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A9" s="4" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="1" t="s">
         <v>185</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A15" s="4" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="272" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B16" s="5" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="138" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B17" s="5" t="s">
+    <row r="17" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="119" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B18" s="5" t="s">
+    <row r="18" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="193" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B19" s="5" t="s">
+    <row r="19" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="238" x14ac:dyDescent="0.2">
-      <c r="A20" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B20" s="5" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>32</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="183" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B21" s="5" t="s">
+    <row r="21" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>34</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="306" x14ac:dyDescent="0.2">
-      <c r="A22" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B22" s="5" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
-      <c r="A23" s="4" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="272" x14ac:dyDescent="0.2">
-      <c r="A24" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B24" s="5" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="255" x14ac:dyDescent="0.2">
-      <c r="A25" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B25" s="5" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="221" x14ac:dyDescent="0.2">
-      <c r="A26" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B26" s="5" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
-      <c r="A27" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B27" s="5" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="388" x14ac:dyDescent="0.2">
-      <c r="A28" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B28" s="5" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="187" x14ac:dyDescent="0.2">
-      <c r="A29" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B29" s="5" t="s">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="204" x14ac:dyDescent="0.2">
-      <c r="A30" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B30" s="5" t="s">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>52</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="238" x14ac:dyDescent="0.2">
-      <c r="A31" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B31" s="5" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>54</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="221" x14ac:dyDescent="0.2">
-      <c r="A32" s="4" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="1" t="s">
         <v>57</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="153" x14ac:dyDescent="0.2">
-      <c r="A33" s="4" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B33" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="85" x14ac:dyDescent="0.2">
-      <c r="A34" s="4" t="s">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="1" t="s">
         <v>58</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="255" x14ac:dyDescent="0.2">
-      <c r="A35" s="4" t="s">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="1" t="s">
         <v>60</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
-      <c r="A36" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B36" s="5" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
-      <c r="A37" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B37" s="5" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="289" x14ac:dyDescent="0.2">
-      <c r="A38" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B38" s="5" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>66</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A39" s="4" t="s">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="B39" s="1" t="s">
         <v>68</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="238" x14ac:dyDescent="0.2">
-      <c r="A40" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B40" s="5" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>70</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="388" x14ac:dyDescent="0.2">
-      <c r="A41" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B41" s="5" t="s">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="255" x14ac:dyDescent="0.2">
-      <c r="A42" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B42" s="5" t="s">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>73</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A43" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B43" s="5" t="s">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B43" s="1" t="s">
         <v>75</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
-      <c r="A44" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B44" s="5" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>77</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="289" x14ac:dyDescent="0.2">
-      <c r="A45" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B45" s="5" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>79</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A46" s="4" t="s">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B46" s="1" t="s">
         <v>80</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="221" x14ac:dyDescent="0.2">
-      <c r="A47" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B47" s="5" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B47" s="1" t="s">
         <v>83</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
-      <c r="A48" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B48" s="5" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B48" s="1" t="s">
         <v>85</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="170" x14ac:dyDescent="0.2">
-      <c r="A49" s="4" t="s">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B49" s="1" t="s">
         <v>87</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
-      <c r="A50" s="4" t="s">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="B50" s="5" t="s">
+      <c r="B50" s="1" t="s">
         <v>89</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="85" x14ac:dyDescent="0.2">
-      <c r="A51" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B51" s="5" t="s">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B51" s="1" t="s">
         <v>91</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="136" x14ac:dyDescent="0.2">
-      <c r="A52" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B52" s="5" t="s">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B52" s="1" t="s">
         <v>93</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="170" x14ac:dyDescent="0.2">
-      <c r="A53" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B53" s="5" t="s">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B53" s="1" t="s">
         <v>95</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="255" x14ac:dyDescent="0.2">
-      <c r="A54" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B54" s="5" t="s">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B54" s="1" t="s">
         <v>97</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="289" x14ac:dyDescent="0.2">
-      <c r="A55" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B55" s="5" t="s">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B55" s="1" t="s">
         <v>99</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="187" x14ac:dyDescent="0.2">
-      <c r="A56" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B56" s="5" t="s">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B56" s="1" t="s">
         <v>101</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="238" x14ac:dyDescent="0.2">
-      <c r="A57" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B57" s="5" t="s">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B57" s="1" t="s">
         <v>103</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="356" x14ac:dyDescent="0.2">
-      <c r="A58" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B58" s="5" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B58" s="1" t="s">
         <v>105</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="289" x14ac:dyDescent="0.2">
-      <c r="A59" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B59" s="5" t="s">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B59" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="323" x14ac:dyDescent="0.2">
-      <c r="A60" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B60" s="5" t="s">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>109</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
-      <c r="A61" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B61" s="5" t="s">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>111</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="409.5" x14ac:dyDescent="0.2">
-      <c r="A62" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B62" s="5" t="s">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B62" s="1" t="s">
         <v>113</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="63" spans="1:3" ht="289" x14ac:dyDescent="0.2">
-      <c r="A63" s="4" t="s">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="B63" s="5" t="s">
+      <c r="B63" s="1" t="s">
         <v>115</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="187" x14ac:dyDescent="0.2">
-      <c r="A64" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B64" s="5" t="s">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B64" s="1" t="s">
         <v>117</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A65" s="4" t="s">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B65" s="5" t="s">
+      <c r="B65" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="C65" s="3" t="s">
+      <c r="C65" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A66" s="4" t="s">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B66" s="5" t="s">
+      <c r="B66" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C66" s="3" t="s">
+      <c r="C66" s="1" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A67" s="4" t="s">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B67" s="5" t="s">
+      <c r="B67" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="C67" s="3" t="s">
+      <c r="C67" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="68" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A68" s="4" t="s">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B68" s="5" t="s">
+      <c r="B68" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="C68" s="3" t="s">
+      <c r="C68" s="1" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="69" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A69" s="4" t="s">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B69" s="5" t="s">
+      <c r="B69" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="C69" s="3" t="s">
+      <c r="C69" s="1" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="70" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A70" s="4" t="s">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B70" s="5" t="s">
+      <c r="B70" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="C70" s="3" t="s">
+      <c r="C70" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="71" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A71" s="4" t="s">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B71" s="5" t="s">
+      <c r="B71" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="C71" s="3" t="s">
+      <c r="C71" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="72" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A72" s="4" t="s">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B72" s="5" t="s">
+      <c r="B72" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C72" s="3" t="s">
+      <c r="C72" s="1" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A73" s="4" t="s">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B73" s="5" t="s">
+      <c r="B73" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C73" s="3" t="s">
+      <c r="C73" s="1" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A74" s="4" t="s">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B74" s="5" t="s">
+      <c r="B74" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C74" s="3" t="s">
+      <c r="C74" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="75" spans="1:3" ht="85" x14ac:dyDescent="0.2">
-      <c r="A75" s="4" t="s">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A75" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B75" s="5" t="s">
+      <c r="B75" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C75" s="3" t="s">
+      <c r="C75" s="1" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="85" x14ac:dyDescent="0.2">
-      <c r="A76" s="4" t="s">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A76" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B76" s="5" t="s">
+      <c r="B76" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C76" s="3" t="s">
+      <c r="C76" s="1" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="77" spans="1:3" ht="85" x14ac:dyDescent="0.2">
-      <c r="A77" s="4" t="s">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A77" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B77" s="5" t="s">
+      <c r="B77" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C77" s="3" t="s">
+      <c r="C77" s="1" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="85" x14ac:dyDescent="0.2">
-      <c r="A78" s="4" t="s">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A78" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B78" s="5" t="s">
+      <c r="B78" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="C78" s="3" t="s">
+      <c r="C78" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="79" spans="1:3" ht="68" x14ac:dyDescent="0.2">
-      <c r="A79" s="4" t="s">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A79" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B79" s="5" t="s">
+      <c r="B79" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="C79" s="3" t="s">
+      <c r="C79" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A80" s="4" t="s">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A80" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B80" s="5" t="s">
+      <c r="B80" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="C80" s="3" t="s">
+      <c r="C80" s="1" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A81" s="4" t="s">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A81" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B81" s="5" t="s">
+      <c r="B81" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C81" s="3" t="s">
+      <c r="C81" s="1" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A82" s="4" t="s">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A82" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B82" s="5" t="s">
+      <c r="B82" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="C82" s="3" t="s">
+      <c r="C82" s="1" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="83" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A83" s="4" t="s">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A83" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B83" s="5" t="s">
+      <c r="B83" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="C83" s="3" t="s">
+      <c r="C83" s="1" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="84" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A84" s="4" t="s">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A84" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B84" s="5" t="s">
+      <c r="B84" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="C84" s="3" t="s">
+      <c r="C84" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A85" s="4" t="s">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A85" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B85" s="5" t="s">
+      <c r="B85" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="C85" s="3" t="s">
+      <c r="C85" s="1" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="86" spans="1:3" ht="136" x14ac:dyDescent="0.2">
-      <c r="A86" s="4" t="s">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A86" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B86" s="5" t="s">
+      <c r="B86" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="C86" s="3" t="s">
+      <c r="C86" s="1" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="87" spans="1:3" ht="136" x14ac:dyDescent="0.2">
-      <c r="A87" s="4" t="s">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A87" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B87" s="5" t="s">
+      <c r="B87" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="C87" s="3" t="s">
+      <c r="C87" s="1" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="88" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A88" s="4" t="s">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A88" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B88" s="5" t="s">
+      <c r="B88" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="C88" s="3" t="s">
+      <c r="C88" s="1" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="89" spans="1:3" ht="68" x14ac:dyDescent="0.2">
-      <c r="A89" s="4" t="s">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A89" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B89" s="5" t="s">
+      <c r="B89" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C89" s="3" t="s">
+      <c r="C89" s="1" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="90" spans="1:3" ht="136" x14ac:dyDescent="0.2">
-      <c r="A90" s="4" t="s">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A90" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="B90" s="5" t="s">
+      <c r="B90" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="C90" s="3" t="s">
+      <c r="C90" s="1" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="91" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A91" s="4" t="s">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A91" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="B91" s="5" t="s">
+      <c r="B91" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="C91" s="3" t="s">
+      <c r="C91" s="1" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="92" spans="1:3" ht="85" x14ac:dyDescent="0.2">
-      <c r="A92" s="4" t="s">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A92" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="B92" s="5" t="s">
+      <c r="B92" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="C92" s="3" t="s">
+      <c r="C92" s="1" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="93" spans="1:3" ht="85" x14ac:dyDescent="0.2">
-      <c r="A93" s="4" t="s">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A93" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="B93" s="5" t="s">
+      <c r="B93" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="C93" s="3" t="s">
+      <c r="C93" s="1" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="94" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A94" s="4" t="s">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A94" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="B94" s="5" t="s">
+      <c r="B94" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="C94" s="3" t="s">
+      <c r="C94" s="1" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A95" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B95" s="4" t="s">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A95" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B95" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="C95" s="3" t="s">
+      <c r="C95" s="1" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="96" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A96" s="4" t="s">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A96" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="B96" s="4" t="s">
+      <c r="B96" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="C96" s="3" t="s">
+      <c r="C96" s="1" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="97" spans="1:3" ht="170" x14ac:dyDescent="0.2">
-      <c r="A97" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B97" s="4" t="s">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A97" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B97" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="C97" s="3" t="s">
+      <c r="C97" s="1" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="98" spans="1:3" ht="238" x14ac:dyDescent="0.2">
-      <c r="A98" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B98" s="4" t="s">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A98" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B98" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="C98" s="3" t="s">
+      <c r="C98" s="1" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="99" spans="1:3" ht="153" x14ac:dyDescent="0.2">
-      <c r="A99" s="4" t="s">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A99" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="B99" s="4" t="s">
+      <c r="B99" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="C99" s="3" t="s">
+      <c r="C99" s="1" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="100" spans="1:3" ht="136" x14ac:dyDescent="0.2">
-      <c r="A100" s="4" t="s">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A100" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B100" s="4" t="s">
+      <c r="B100" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="C100" s="3" t="s">
+      <c r="C100" s="1" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="101" spans="1:3" ht="204" x14ac:dyDescent="0.2">
-      <c r="A101" s="4" t="s">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A101" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B101" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="C101" s="3" t="s">
+      <c r="C101" s="1" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="102" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A102" s="4" t="s">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A102" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="B102" s="4" t="s">
+      <c r="B102" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A103" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C103" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="C102" s="3" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A103" s="4" t="s">
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A104" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A105" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A106" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A107" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A108" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A109" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A110" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A111" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="B103" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="C103" s="3" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" ht="204" x14ac:dyDescent="0.2">
-      <c r="A104" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B104" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="C104" s="3" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3" ht="170" x14ac:dyDescent="0.2">
-      <c r="A105" s="4" t="s">
+      <c r="B111" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A112" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A113" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A114" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A115" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A116" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B116" t="s">
+        <v>241</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A117" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B117" t="s">
+        <v>243</v>
+      </c>
+      <c r="C117" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A118" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B118" t="s">
+        <v>245</v>
+      </c>
+      <c r="C118" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A119" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B119" t="s">
+        <v>247</v>
+      </c>
+      <c r="C119" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A120" t="s">
+        <v>183</v>
+      </c>
+      <c r="B120" t="s">
+        <v>249</v>
+      </c>
+      <c r="C120" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A121" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="B105" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="C105" s="3" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" ht="255" x14ac:dyDescent="0.2">
-      <c r="A106" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B106" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="C106" s="3" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" ht="119" x14ac:dyDescent="0.2">
-      <c r="A107" s="4" t="s">
+      <c r="B121" t="s">
+        <v>251</v>
+      </c>
+      <c r="C121" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A122" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B122" t="s">
+        <v>253</v>
+      </c>
+      <c r="C122" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A123" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="B107" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="C107" s="3" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A108" s="4" t="s">
+      <c r="B123" t="s">
+        <v>255</v>
+      </c>
+      <c r="C123" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A124" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B124" t="s">
+        <v>257</v>
+      </c>
+      <c r="C124" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A125" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="B108" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="C108" s="3" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3" ht="170" x14ac:dyDescent="0.2">
-      <c r="A109" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B109" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="C109" s="3" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3" ht="204" x14ac:dyDescent="0.2">
-      <c r="A110" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B110" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="C110" s="3" t="s">
-        <v>229</v>
+      <c r="B125" t="s">
+        <v>259</v>
+      </c>
+      <c r="C125" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A126" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="C126" s="3" t="s">
+        <v>262</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>